<commit_message>
Add angle calculations and local axes for bars
Implemented methods in core/barra.py to calculate alpha, beta, and gamma angles, as well as local axes for bars. Updated carga_puntual.py to use new rotation attribute names. Added a utility script (testeos.py) to generate and export bar angle and axis data to Excel for verification. Minor update in io/carga_barra.py to ensure bar length is calculated from node coordinates. Added new Excel files for angle and test data.
</commit_message>
<xml_diff>
--- a/io/Datos_template.xlsx
+++ b/io/Datos_template.xlsx
@@ -788,10 +788,10 @@
         <v>3</v>
       </c>
       <c r="C5" s="16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D5" s="17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" s="16">
         <v>1</v>
@@ -1152,10 +1152,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="6">
+        <v>3</v>
+      </c>
+      <c r="C3" s="6">
         <v>2</v>
-      </c>
-      <c r="C3" s="6">
-        <v>3</v>
       </c>
       <c r="D3" s="6">
         <v>200</v>
@@ -1176,7 +1176,7 @@
         <v>234</v>
       </c>
       <c r="J3" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>

</xml_diff>